<commit_message>
fix: restaurar JSON de stock limpio y regenerar reportes (sin marcas de conflicto)
</commit_message>
<xml_diff>
--- a/frontend/public/reports/StockPulse_PELOTAS.xlsx
+++ b/frontend/public/reports/StockPulse_PELOTAS.xlsx
@@ -52,475 +52,475 @@
     <t>FUTBOL CUERO TERMOSELLADA PRECISION #5</t>
   </si>
   <si>
+    <t>✗ AGOTADO</t>
+  </si>
+  <si>
     <t>016726</t>
   </si>
   <si>
     <t>FUTBOL CUERO TERMOSELLADA DUPLO #5</t>
   </si>
   <si>
+    <t>016727</t>
+  </si>
+  <si>
+    <t>7754807167277</t>
+  </si>
+  <si>
+    <t>FUTBOL CUERO TERMOSELLADA LEAGUE #5</t>
+  </si>
+  <si>
+    <t>016756</t>
+  </si>
+  <si>
+    <t>FUTBOL CUERO TERMOSELLADA LEAGUE #4</t>
+  </si>
+  <si>
+    <t>016755</t>
+  </si>
+  <si>
+    <t>FUTBOL CUERO TERMOSELLADA PRESTIGE #5</t>
+  </si>
+  <si>
+    <t>016757</t>
+  </si>
+  <si>
+    <t>7754807167574</t>
+  </si>
+  <si>
+    <t>FUTBOL CUERO TERMOSELLADA PERU #5</t>
+  </si>
+  <si>
+    <t>016760</t>
+  </si>
+  <si>
+    <t>7754807167604</t>
+  </si>
+  <si>
+    <t>FUTBOL CUERO TERMOSELLADA PERU #4</t>
+  </si>
+  <si>
+    <t>016758</t>
+  </si>
+  <si>
+    <t>FUTBOL CUERO TERMOSELLADA ARGENTINA #5</t>
+  </si>
+  <si>
+    <t>016761</t>
+  </si>
+  <si>
+    <t>7754807167611</t>
+  </si>
+  <si>
+    <t>FUTBOL CUERO TERMOSELLADA ARGENTINA #4</t>
+  </si>
+  <si>
+    <t>016759</t>
+  </si>
+  <si>
+    <t>FUTBOL CUERO TERMOSELLADA BRASIL #5</t>
+  </si>
+  <si>
+    <t>016762</t>
+  </si>
+  <si>
+    <t>7754807167628</t>
+  </si>
+  <si>
+    <t>FUTBOL CUERO TERMOSELLADA BRASIL #4</t>
+  </si>
+  <si>
+    <t>016706</t>
+  </si>
+  <si>
+    <t>7754807167062</t>
+  </si>
+  <si>
+    <t>FUTBOL CUERO TERMOSELLADA BLANQUIRROJA #5</t>
+  </si>
+  <si>
+    <t>016708</t>
+  </si>
+  <si>
+    <t>7754807167086</t>
+  </si>
+  <si>
+    <t>FUTBOL CUERO TERMOSELLADA PEGASUS #5</t>
+  </si>
+  <si>
+    <t>014375</t>
+  </si>
+  <si>
+    <t>7754807143752</t>
+  </si>
+  <si>
+    <t>FUTSAL CUERO VULC #3.5</t>
+  </si>
+  <si>
+    <t>016766</t>
+  </si>
+  <si>
+    <t>FUTSAL TERMOSELLADA ALEGRO</t>
+  </si>
+  <si>
+    <t>016767</t>
+  </si>
+  <si>
+    <t>FUTBOL VULCANIZADA PREMIER1 #5</t>
+  </si>
+  <si>
+    <t>016768</t>
+  </si>
+  <si>
+    <t>FUTBOL VULCANIZADA PREMIER2 #5</t>
+  </si>
+  <si>
+    <t>016769</t>
+  </si>
+  <si>
+    <t>FUTBOL VULCANIZADA PREMIER3 #5</t>
+  </si>
+  <si>
+    <t>016770</t>
+  </si>
+  <si>
+    <t>FUTBOL VULCANIZADA PREMIER4 #5</t>
+  </si>
+  <si>
+    <t>016771</t>
+  </si>
+  <si>
+    <t>FUTBOL VULCANIZADA PREMIER1 #4</t>
+  </si>
+  <si>
+    <t>016743</t>
+  </si>
+  <si>
+    <t>FUTBOL TPU PER2 CUP24 #5</t>
+  </si>
+  <si>
+    <t>016744</t>
+  </si>
+  <si>
+    <t>FUTBOL TPU BRA2 CUP24 #5</t>
+  </si>
+  <si>
+    <t>016745</t>
+  </si>
+  <si>
+    <t>FUTBOL TPU ARG2 CUP24 #5</t>
+  </si>
+  <si>
+    <t>016746</t>
+  </si>
+  <si>
+    <t>FUTBOL TPU FLAGS CUP24 #5</t>
+  </si>
+  <si>
+    <t>016747</t>
+  </si>
+  <si>
+    <t>VOLEY PU LIGA1</t>
+  </si>
+  <si>
+    <t>016748</t>
+  </si>
+  <si>
+    <t>VOLEY PU LIGA2</t>
+  </si>
+  <si>
+    <t>016729</t>
+  </si>
+  <si>
+    <t>VOLEY CUERO COSIDO FLORES</t>
+  </si>
+  <si>
+    <t>016731</t>
+  </si>
+  <si>
+    <t>VOLEY CUP CUERO COSIDO CELESTE AMARILLO ROSADO</t>
+  </si>
+  <si>
+    <t>016728</t>
+  </si>
+  <si>
+    <t>VOLEY CUERO COSIDO FOLK</t>
+  </si>
+  <si>
+    <t>016730</t>
+  </si>
+  <si>
+    <t>7754807167307</t>
+  </si>
+  <si>
+    <t>VOLEY CUERO COSIDO FOLK GRAFITTI</t>
+  </si>
+  <si>
+    <t>016788</t>
+  </si>
+  <si>
+    <t>7754807167888</t>
+  </si>
+  <si>
+    <t>VOLEY CUERO COSIDO CREW</t>
+  </si>
+  <si>
+    <t>016737</t>
+  </si>
+  <si>
+    <t>VOLEY CELULAR PWR1</t>
+  </si>
+  <si>
+    <t>016738</t>
+  </si>
+  <si>
+    <t>VOLEY CELULAR PWR2</t>
+  </si>
+  <si>
+    <t>016739</t>
+  </si>
+  <si>
+    <t>VOLEY CELULAR PWR3</t>
+  </si>
+  <si>
+    <t>016004</t>
+  </si>
+  <si>
+    <t>7754807160049</t>
+  </si>
+  <si>
+    <t>FUTBOL GOMA SPARTANO #3</t>
+  </si>
+  <si>
+    <t>015938</t>
+  </si>
+  <si>
+    <t>7754807159388</t>
+  </si>
+  <si>
+    <t>FUTBOL GOMA FREE #5</t>
+  </si>
+  <si>
+    <t>016678</t>
+  </si>
+  <si>
+    <t>7754807166782</t>
+  </si>
+  <si>
+    <t>FUTBOL GOMA URBAN #5</t>
+  </si>
+  <si>
+    <t>016724</t>
+  </si>
+  <si>
+    <t>7754807167246</t>
+  </si>
+  <si>
+    <t>FUTBOL GOMA SPECTRE #5</t>
+  </si>
+  <si>
+    <t>016783</t>
+  </si>
+  <si>
+    <t>7754807167833</t>
+  </si>
+  <si>
+    <t>FUTBOL GOMA INVICTUS  #5</t>
+  </si>
+  <si>
+    <t>014323</t>
+  </si>
+  <si>
+    <t>7754807143233</t>
+  </si>
+  <si>
+    <t>FUTBOL GOMA PAISES BLANCO #5</t>
+  </si>
+  <si>
+    <t>014796</t>
+  </si>
+  <si>
+    <t>7754807147965</t>
+  </si>
+  <si>
+    <t>FUTBOL GOMA TEAM #5</t>
+  </si>
+  <si>
+    <t>011883</t>
+  </si>
+  <si>
+    <t>7754807118835</t>
+  </si>
+  <si>
+    <t>FUTBOL GOMA PAISES COLORES #5</t>
+  </si>
+  <si>
+    <t>016657</t>
+  </si>
+  <si>
+    <t>7754807166577</t>
+  </si>
+  <si>
+    <t>VOLEY GOMA BUTTERFLY</t>
+  </si>
+  <si>
+    <t>015936</t>
+  </si>
+  <si>
+    <t>7754807159364</t>
+  </si>
+  <si>
+    <t>VOLEY VINIBALL GOMA MULTICOLOR</t>
+  </si>
+  <si>
+    <t>014268</t>
+  </si>
+  <si>
+    <t>7754807142687</t>
+  </si>
+  <si>
+    <t>VOLEY VINIBALL GOMA TRICOLOR</t>
+  </si>
+  <si>
+    <t>016784</t>
+  </si>
+  <si>
+    <t>7754807167840</t>
+  </si>
+  <si>
+    <t>VOLEY GOMA FLORES2</t>
+  </si>
+  <si>
+    <t>016786</t>
+  </si>
+  <si>
+    <t>7754807167864</t>
+  </si>
+  <si>
+    <t>VOLEY GOMA FRUTAS2</t>
+  </si>
+  <si>
+    <t>015939</t>
+  </si>
+  <si>
+    <t>7754807159395</t>
+  </si>
+  <si>
+    <t>VOLEY VINIBALL GOMA FOLK</t>
+  </si>
+  <si>
+    <t>016785</t>
+  </si>
+  <si>
+    <t>7754807167857</t>
+  </si>
+  <si>
+    <t>VOLEY GOMA MARIPOSAS</t>
+  </si>
+  <si>
+    <t>016787</t>
+  </si>
+  <si>
+    <t>7754807167871</t>
+  </si>
+  <si>
+    <t>VOLEY GOMA URBANA</t>
+  </si>
+  <si>
+    <t>016672</t>
+  </si>
+  <si>
+    <t>7754807166720</t>
+  </si>
+  <si>
+    <t>BASQUET GOMA #3 SONRISAS</t>
+  </si>
+  <si>
+    <t>014271</t>
+  </si>
+  <si>
+    <t>7754807142717</t>
+  </si>
+  <si>
+    <t>BASQUET GOMA #3 NARANJA</t>
+  </si>
+  <si>
+    <t>014270</t>
+  </si>
+  <si>
+    <t>7754807111638</t>
+  </si>
+  <si>
+    <t>BASQUET GOMA #5 NARANJA</t>
+  </si>
+  <si>
+    <t>014277</t>
+  </si>
+  <si>
+    <t>7754807142779</t>
+  </si>
+  <si>
+    <t>BASQUET GOMA #7 NARANJA</t>
+  </si>
+  <si>
+    <t>015933</t>
+  </si>
+  <si>
+    <t>7754807159333</t>
+  </si>
+  <si>
+    <t>BASQUET GOMA #7 PERU</t>
+  </si>
+  <si>
+    <t>016676</t>
+  </si>
+  <si>
+    <t>7754807166768</t>
+  </si>
+  <si>
+    <t>BASQUET GOMA #5 GALAXY</t>
+  </si>
+  <si>
+    <t>016675</t>
+  </si>
+  <si>
+    <t>7754807166751</t>
+  </si>
+  <si>
+    <t>BASQUET GOMA #7 GALAXY</t>
+  </si>
+  <si>
+    <t>016752</t>
+  </si>
+  <si>
+    <t>BASQUET GOMA #5 LEGACY</t>
+  </si>
+  <si>
+    <t>016750</t>
+  </si>
+  <si>
+    <t>BASQUET GOMA #7 LEGACY</t>
+  </si>
+  <si>
+    <t>016751</t>
+  </si>
+  <si>
+    <t>BASQUET GOMA #5 JAM</t>
+  </si>
+  <si>
+    <t>016749</t>
+  </si>
+  <si>
+    <t>BASQUET GOMA #7 JAM</t>
+  </si>
+  <si>
+    <t>016764</t>
+  </si>
+  <si>
+    <t>BALONMANO GOMA #1</t>
+  </si>
+  <si>
     <t>⚠ BAJO</t>
-  </si>
-  <si>
-    <t>016727</t>
-  </si>
-  <si>
-    <t>7754807167277</t>
-  </si>
-  <si>
-    <t>FUTBOL CUERO TERMOSELLADA LEAGUE #5</t>
-  </si>
-  <si>
-    <t>016756</t>
-  </si>
-  <si>
-    <t>FUTBOL CUERO TERMOSELLADA LEAGUE #4</t>
-  </si>
-  <si>
-    <t>016755</t>
-  </si>
-  <si>
-    <t>FUTBOL CUERO TERMOSELLADA PRESTIGE #5</t>
-  </si>
-  <si>
-    <t>✗ AGOTADO</t>
-  </si>
-  <si>
-    <t>016757</t>
-  </si>
-  <si>
-    <t>7754807167574</t>
-  </si>
-  <si>
-    <t>FUTBOL CUERO TERMOSELLADA PERU #5</t>
-  </si>
-  <si>
-    <t>016760</t>
-  </si>
-  <si>
-    <t>7754807167604</t>
-  </si>
-  <si>
-    <t>FUTBOL CUERO TERMOSELLADA PERU #4</t>
-  </si>
-  <si>
-    <t>016758</t>
-  </si>
-  <si>
-    <t>FUTBOL CUERO TERMOSELLADA ARGENTINA #5</t>
-  </si>
-  <si>
-    <t>016761</t>
-  </si>
-  <si>
-    <t>7754807167611</t>
-  </si>
-  <si>
-    <t>FUTBOL CUERO TERMOSELLADA ARGENTINA #4</t>
-  </si>
-  <si>
-    <t>016759</t>
-  </si>
-  <si>
-    <t>FUTBOL CUERO TERMOSELLADA BRASIL #5</t>
-  </si>
-  <si>
-    <t>016762</t>
-  </si>
-  <si>
-    <t>7754807167628</t>
-  </si>
-  <si>
-    <t>FUTBOL CUERO TERMOSELLADA BRASIL #4</t>
-  </si>
-  <si>
-    <t>016706</t>
-  </si>
-  <si>
-    <t>7754807167062</t>
-  </si>
-  <si>
-    <t>FUTBOL CUERO TERMOSELLADA BLANQUIRROJA #5</t>
-  </si>
-  <si>
-    <t>016708</t>
-  </si>
-  <si>
-    <t>7754807167086</t>
-  </si>
-  <si>
-    <t>FUTBOL CUERO TERMOSELLADA PEGASUS #5</t>
-  </si>
-  <si>
-    <t>014375</t>
-  </si>
-  <si>
-    <t>7754807143752</t>
-  </si>
-  <si>
-    <t>FUTSAL CUERO VULC #3.5</t>
-  </si>
-  <si>
-    <t>016766</t>
-  </si>
-  <si>
-    <t>FUTSAL TERMOSELLADA ALEGRO</t>
-  </si>
-  <si>
-    <t>016767</t>
-  </si>
-  <si>
-    <t>FUTBOL VULCANIZADA PREMIER1 #5</t>
-  </si>
-  <si>
-    <t>016768</t>
-  </si>
-  <si>
-    <t>FUTBOL VULCANIZADA PREMIER2 #5</t>
-  </si>
-  <si>
-    <t>016769</t>
-  </si>
-  <si>
-    <t>FUTBOL VULCANIZADA PREMIER3 #5</t>
-  </si>
-  <si>
-    <t>016770</t>
-  </si>
-  <si>
-    <t>FUTBOL VULCANIZADA PREMIER4 #5</t>
-  </si>
-  <si>
-    <t>016771</t>
-  </si>
-  <si>
-    <t>FUTBOL VULCANIZADA PREMIER1 #4</t>
-  </si>
-  <si>
-    <t>016743</t>
-  </si>
-  <si>
-    <t>FUTBOL TPU PER2 CUP24 #5</t>
-  </si>
-  <si>
-    <t>016744</t>
-  </si>
-  <si>
-    <t>FUTBOL TPU BRA2 CUP24 #5</t>
-  </si>
-  <si>
-    <t>016745</t>
-  </si>
-  <si>
-    <t>FUTBOL TPU ARG2 CUP24 #5</t>
-  </si>
-  <si>
-    <t>016746</t>
-  </si>
-  <si>
-    <t>FUTBOL TPU FLAGS CUP24 #5</t>
-  </si>
-  <si>
-    <t>016747</t>
-  </si>
-  <si>
-    <t>VOLEY PU LIGA1</t>
-  </si>
-  <si>
-    <t>016748</t>
-  </si>
-  <si>
-    <t>VOLEY PU LIGA2</t>
-  </si>
-  <si>
-    <t>016729</t>
-  </si>
-  <si>
-    <t>VOLEY CUERO COSIDO FLORES</t>
-  </si>
-  <si>
-    <t>016731</t>
-  </si>
-  <si>
-    <t>VOLEY CUP CUERO COSIDO CELESTE AMARILLO ROSADO</t>
-  </si>
-  <si>
-    <t>016728</t>
-  </si>
-  <si>
-    <t>VOLEY CUERO COSIDO FOLK</t>
-  </si>
-  <si>
-    <t>016730</t>
-  </si>
-  <si>
-    <t>7754807167307</t>
-  </si>
-  <si>
-    <t>VOLEY CUERO COSIDO FOLK GRAFITTI</t>
-  </si>
-  <si>
-    <t>016788</t>
-  </si>
-  <si>
-    <t>7754807167888</t>
-  </si>
-  <si>
-    <t>VOLEY CUERO COSIDO CREW</t>
-  </si>
-  <si>
-    <t>016737</t>
-  </si>
-  <si>
-    <t>VOLEY CELULAR PWR1</t>
-  </si>
-  <si>
-    <t>016738</t>
-  </si>
-  <si>
-    <t>VOLEY CELULAR PWR2</t>
-  </si>
-  <si>
-    <t>016739</t>
-  </si>
-  <si>
-    <t>VOLEY CELULAR PWR3</t>
-  </si>
-  <si>
-    <t>016004</t>
-  </si>
-  <si>
-    <t>7754807160049</t>
-  </si>
-  <si>
-    <t>FUTBOL GOMA SPARTANO #3</t>
-  </si>
-  <si>
-    <t>015938</t>
-  </si>
-  <si>
-    <t>7754807159388</t>
-  </si>
-  <si>
-    <t>FUTBOL GOMA FREE #5</t>
-  </si>
-  <si>
-    <t>016678</t>
-  </si>
-  <si>
-    <t>7754807166782</t>
-  </si>
-  <si>
-    <t>FUTBOL GOMA URBAN #5</t>
-  </si>
-  <si>
-    <t>016724</t>
-  </si>
-  <si>
-    <t>7754807167246</t>
-  </si>
-  <si>
-    <t>FUTBOL GOMA SPECTRE #5</t>
-  </si>
-  <si>
-    <t>016783</t>
-  </si>
-  <si>
-    <t>7754807167833</t>
-  </si>
-  <si>
-    <t>FUTBOL GOMA INVICTUS  #5</t>
-  </si>
-  <si>
-    <t>014323</t>
-  </si>
-  <si>
-    <t>7754807143233</t>
-  </si>
-  <si>
-    <t>FUTBOL GOMA PAISES BLANCO #5</t>
-  </si>
-  <si>
-    <t>014796</t>
-  </si>
-  <si>
-    <t>7754807147965</t>
-  </si>
-  <si>
-    <t>FUTBOL GOMA TEAM #5</t>
-  </si>
-  <si>
-    <t>011883</t>
-  </si>
-  <si>
-    <t>7754807118835</t>
-  </si>
-  <si>
-    <t>FUTBOL GOMA PAISES COLORES #5</t>
-  </si>
-  <si>
-    <t>016657</t>
-  </si>
-  <si>
-    <t>7754807166577</t>
-  </si>
-  <si>
-    <t>VOLEY GOMA BUTTERFLY</t>
-  </si>
-  <si>
-    <t>015936</t>
-  </si>
-  <si>
-    <t>7754807159364</t>
-  </si>
-  <si>
-    <t>VOLEY VINIBALL GOMA MULTICOLOR</t>
-  </si>
-  <si>
-    <t>014268</t>
-  </si>
-  <si>
-    <t>7754807142687</t>
-  </si>
-  <si>
-    <t>VOLEY VINIBALL GOMA TRICOLOR</t>
-  </si>
-  <si>
-    <t>016784</t>
-  </si>
-  <si>
-    <t>7754807167840</t>
-  </si>
-  <si>
-    <t>VOLEY GOMA FLORES2</t>
-  </si>
-  <si>
-    <t>016786</t>
-  </si>
-  <si>
-    <t>7754807167864</t>
-  </si>
-  <si>
-    <t>VOLEY GOMA FRUTAS2</t>
-  </si>
-  <si>
-    <t>015939</t>
-  </si>
-  <si>
-    <t>7754807159395</t>
-  </si>
-  <si>
-    <t>VOLEY VINIBALL GOMA FOLK</t>
-  </si>
-  <si>
-    <t>016785</t>
-  </si>
-  <si>
-    <t>7754807167857</t>
-  </si>
-  <si>
-    <t>VOLEY GOMA MARIPOSAS</t>
-  </si>
-  <si>
-    <t>016787</t>
-  </si>
-  <si>
-    <t>7754807167871</t>
-  </si>
-  <si>
-    <t>VOLEY GOMA URBANA</t>
-  </si>
-  <si>
-    <t>016672</t>
-  </si>
-  <si>
-    <t>7754807166720</t>
-  </si>
-  <si>
-    <t>BASQUET GOMA #3 SONRISAS</t>
-  </si>
-  <si>
-    <t>014271</t>
-  </si>
-  <si>
-    <t>7754807142717</t>
-  </si>
-  <si>
-    <t>BASQUET GOMA #3 NARANJA</t>
-  </si>
-  <si>
-    <t>014270</t>
-  </si>
-  <si>
-    <t>7754807111638</t>
-  </si>
-  <si>
-    <t>BASQUET GOMA #5 NARANJA</t>
-  </si>
-  <si>
-    <t>014277</t>
-  </si>
-  <si>
-    <t>7754807142779</t>
-  </si>
-  <si>
-    <t>BASQUET GOMA #7 NARANJA</t>
-  </si>
-  <si>
-    <t>015933</t>
-  </si>
-  <si>
-    <t>7754807159333</t>
-  </si>
-  <si>
-    <t>BASQUET GOMA #7 PERU</t>
-  </si>
-  <si>
-    <t>016676</t>
-  </si>
-  <si>
-    <t>7754807166768</t>
-  </si>
-  <si>
-    <t>BASQUET GOMA #5 GALAXY</t>
-  </si>
-  <si>
-    <t>016675</t>
-  </si>
-  <si>
-    <t>7754807166751</t>
-  </si>
-  <si>
-    <t>BASQUET GOMA #7 GALAXY</t>
-  </si>
-  <si>
-    <t>016752</t>
-  </si>
-  <si>
-    <t>BASQUET GOMA #5 LEGACY</t>
-  </si>
-  <si>
-    <t>016750</t>
-  </si>
-  <si>
-    <t>BASQUET GOMA #7 LEGACY</t>
-  </si>
-  <si>
-    <t>016751</t>
-  </si>
-  <si>
-    <t>BASQUET GOMA #5 JAM</t>
-  </si>
-  <si>
-    <t>016749</t>
-  </si>
-  <si>
-    <t>BASQUET GOMA #7 JAM</t>
-  </si>
-  <si>
-    <t>016764</t>
-  </si>
-  <si>
-    <t>BALONMANO GOMA #1</t>
   </si>
   <si>
     <t>016765</t>
@@ -1712,12 +1712,12 @@
     </font>
     <font>
       <b/>
-      <color rgb="FFD97706"/>
+      <color rgb="FFDC2626"/>
       <sz val="12"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFDC2626"/>
+      <color rgb="FFD97706"/>
       <sz val="12"/>
     </font>
   </fonts>
@@ -1740,12 +1740,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFEF3C7"/>
+        <fgColor rgb="FFFEE2E2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFEE2E2"/>
+        <fgColor rgb="FFFEF3C7"/>
       </patternFill>
     </fill>
   </fills>
@@ -2196,11 +2196,11 @@
       <c r="E3">
         <v>24</v>
       </c>
-      <c r="F3" s="2">
-        <v>2050</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>10</v>
+      <c r="F3" s="4">
+        <v>0</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -2208,22 +2208,22 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C4" t="s">
         <v>8</v>
       </c>
       <c r="D4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E4">
         <v>24</v>
       </c>
       <c r="F4" s="4">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -2242,11 +2242,11 @@
       <c r="E5">
         <v>24</v>
       </c>
-      <c r="F5" s="2">
-        <v>3800</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>10</v>
+      <c r="F5" s="4">
+        <v>0</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -2265,11 +2265,11 @@
       <c r="E6">
         <v>24</v>
       </c>
-      <c r="F6" s="2">
-        <v>606</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>10</v>
+      <c r="F6" s="4">
+        <v>0</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -2288,11 +2288,11 @@
       <c r="E7">
         <v>24</v>
       </c>
-      <c r="F7" s="6">
-        <v>0</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>23</v>
+      <c r="F7" s="4">
+        <v>0</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -2300,22 +2300,22 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" t="s">
         <v>24</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>25</v>
-      </c>
-      <c r="D8" t="s">
-        <v>26</v>
       </c>
       <c r="E8">
         <v>24</v>
       </c>
-      <c r="F8" s="2">
-        <v>4742</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>10</v>
+      <c r="F8" s="4">
+        <v>0</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -2323,22 +2323,22 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" t="s">
         <v>27</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>28</v>
-      </c>
-      <c r="D9" t="s">
-        <v>29</v>
       </c>
       <c r="E9">
         <v>24</v>
       </c>
-      <c r="F9" s="2">
-        <v>1463</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>10</v>
+      <c r="F9" s="4">
+        <v>0</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -2346,22 +2346,22 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C10" t="s">
         <v>8</v>
       </c>
       <c r="D10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E10">
         <v>24</v>
       </c>
-      <c r="F10" s="2">
-        <v>1496</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>10</v>
+      <c r="F10" s="4">
+        <v>0</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -2369,22 +2369,22 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" t="s">
         <v>32</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>33</v>
-      </c>
-      <c r="D11" t="s">
-        <v>34</v>
       </c>
       <c r="E11">
         <v>24</v>
       </c>
-      <c r="F11" s="2">
-        <v>180</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>10</v>
+      <c r="F11" s="4">
+        <v>0</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -2392,22 +2392,22 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C12" t="s">
         <v>8</v>
       </c>
       <c r="D12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E12">
         <v>24</v>
       </c>
-      <c r="F12" s="2">
-        <v>1426</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>10</v>
+      <c r="F12" s="4">
+        <v>0</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -2415,22 +2415,22 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" t="s">
         <v>37</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>38</v>
-      </c>
-      <c r="D13" t="s">
-        <v>39</v>
       </c>
       <c r="E13">
         <v>24</v>
       </c>
-      <c r="F13" s="2">
-        <v>168</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>10</v>
+      <c r="F13" s="4">
+        <v>0</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -2438,22 +2438,22 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" t="s">
         <v>40</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>41</v>
-      </c>
-      <c r="D14" t="s">
-        <v>42</v>
       </c>
       <c r="E14">
         <v>36</v>
       </c>
-      <c r="F14" s="2">
-        <v>182</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>10</v>
+      <c r="F14" s="4">
+        <v>0</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -2461,22 +2461,22 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
+        <v>42</v>
+      </c>
+      <c r="C15" t="s">
         <v>43</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>44</v>
-      </c>
-      <c r="D15" t="s">
-        <v>45</v>
       </c>
       <c r="E15">
         <v>36</v>
       </c>
       <c r="F15" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -2484,22 +2484,22 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" t="s">
         <v>46</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>47</v>
-      </c>
-      <c r="D16" t="s">
-        <v>48</v>
       </c>
       <c r="E16">
         <v>36</v>
       </c>
-      <c r="F16" s="2">
-        <v>1012</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>10</v>
+      <c r="F16" s="4">
+        <v>0</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -2507,22 +2507,22 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C17" t="s">
         <v>8</v>
       </c>
       <c r="D17" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E17">
         <v>24</v>
       </c>
       <c r="F17" s="4">
-        <v>76</v>
+        <v>0</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -2530,22 +2530,22 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C18" t="s">
         <v>8</v>
       </c>
       <c r="D18" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E18">
         <v>36</v>
       </c>
-      <c r="F18" s="6">
-        <v>0</v>
-      </c>
-      <c r="G18" s="7" t="s">
-        <v>23</v>
+      <c r="F18" s="4">
+        <v>0</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -2553,22 +2553,22 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C19" t="s">
         <v>8</v>
       </c>
       <c r="D19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E19">
         <v>36</v>
       </c>
-      <c r="F19" s="2">
-        <v>3828</v>
-      </c>
-      <c r="G19" s="3" t="s">
-        <v>10</v>
+      <c r="F19" s="4">
+        <v>0</v>
+      </c>
+      <c r="G19" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -2576,22 +2576,22 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C20" t="s">
         <v>8</v>
       </c>
       <c r="D20" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E20">
         <v>36</v>
       </c>
-      <c r="F20" s="2">
-        <v>3206</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>10</v>
+      <c r="F20" s="4">
+        <v>0</v>
+      </c>
+      <c r="G20" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -2599,22 +2599,22 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C21" t="s">
         <v>8</v>
       </c>
       <c r="D21" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E21">
         <v>36</v>
       </c>
-      <c r="F21" s="2">
-        <v>8229</v>
-      </c>
-      <c r="G21" s="3" t="s">
-        <v>10</v>
+      <c r="F21" s="4">
+        <v>0</v>
+      </c>
+      <c r="G21" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -2622,22 +2622,22 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C22" t="s">
         <v>8</v>
       </c>
       <c r="D22" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E22">
         <v>36</v>
       </c>
-      <c r="F22" s="2">
-        <v>1330</v>
-      </c>
-      <c r="G22" s="3" t="s">
-        <v>10</v>
+      <c r="F22" s="4">
+        <v>0</v>
+      </c>
+      <c r="G22" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -2645,22 +2645,22 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C23" t="s">
         <v>8</v>
       </c>
       <c r="D23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E23">
         <v>48</v>
       </c>
-      <c r="F23" s="6">
-        <v>0</v>
-      </c>
-      <c r="G23" s="7" t="s">
-        <v>23</v>
+      <c r="F23" s="4">
+        <v>0</v>
+      </c>
+      <c r="G23" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -2668,22 +2668,22 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C24" t="s">
         <v>8</v>
       </c>
       <c r="D24" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E24">
         <v>48</v>
       </c>
-      <c r="F24" s="6">
-        <v>0</v>
-      </c>
-      <c r="G24" s="7" t="s">
-        <v>23</v>
+      <c r="F24" s="4">
+        <v>0</v>
+      </c>
+      <c r="G24" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -2691,22 +2691,22 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C25" t="s">
         <v>8</v>
       </c>
       <c r="D25" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E25">
         <v>48</v>
       </c>
-      <c r="F25" s="6">
-        <v>0</v>
-      </c>
-      <c r="G25" s="7" t="s">
-        <v>23</v>
+      <c r="F25" s="4">
+        <v>0</v>
+      </c>
+      <c r="G25" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -2714,22 +2714,22 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C26" t="s">
         <v>8</v>
       </c>
       <c r="D26" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E26">
         <v>48</v>
       </c>
       <c r="F26" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -2737,22 +2737,22 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C27" t="s">
         <v>8</v>
       </c>
       <c r="D27" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E27">
         <v>36</v>
       </c>
-      <c r="F27" s="6">
-        <v>0</v>
-      </c>
-      <c r="G27" s="7" t="s">
-        <v>23</v>
+      <c r="F27" s="4">
+        <v>0</v>
+      </c>
+      <c r="G27" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -2760,22 +2760,22 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C28" t="s">
         <v>8</v>
       </c>
       <c r="D28" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E28">
         <v>36</v>
       </c>
       <c r="F28" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -2783,22 +2783,22 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C29" t="s">
         <v>8</v>
       </c>
       <c r="D29" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E29">
         <v>50</v>
       </c>
-      <c r="F29" s="2">
-        <v>3043</v>
-      </c>
-      <c r="G29" s="3" t="s">
-        <v>10</v>
+      <c r="F29" s="4">
+        <v>0</v>
+      </c>
+      <c r="G29" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
@@ -2806,22 +2806,22 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C30" t="s">
         <v>8</v>
       </c>
       <c r="D30" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E30">
         <v>50</v>
       </c>
-      <c r="F30" s="6">
-        <v>0</v>
-      </c>
-      <c r="G30" s="7" t="s">
-        <v>23</v>
+      <c r="F30" s="4">
+        <v>0</v>
+      </c>
+      <c r="G30" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
@@ -2829,22 +2829,22 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C31" t="s">
         <v>8</v>
       </c>
       <c r="D31" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E31">
         <v>50</v>
       </c>
-      <c r="F31" s="6">
-        <v>0</v>
-      </c>
-      <c r="G31" s="7" t="s">
-        <v>23</v>
+      <c r="F31" s="4">
+        <v>0</v>
+      </c>
+      <c r="G31" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
@@ -2852,22 +2852,22 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
+        <v>78</v>
+      </c>
+      <c r="C32" t="s">
         <v>79</v>
       </c>
-      <c r="C32" t="s">
+      <c r="D32" t="s">
         <v>80</v>
-      </c>
-      <c r="D32" t="s">
-        <v>81</v>
       </c>
       <c r="E32">
         <v>50</v>
       </c>
-      <c r="F32" s="2">
-        <v>3505</v>
-      </c>
-      <c r="G32" s="3" t="s">
-        <v>10</v>
+      <c r="F32" s="4">
+        <v>0</v>
+      </c>
+      <c r="G32" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
@@ -2875,22 +2875,22 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
+        <v>81</v>
+      </c>
+      <c r="C33" t="s">
         <v>82</v>
       </c>
-      <c r="C33" t="s">
+      <c r="D33" t="s">
         <v>83</v>
-      </c>
-      <c r="D33" t="s">
-        <v>84</v>
       </c>
       <c r="E33">
         <v>50</v>
       </c>
-      <c r="F33" s="2">
-        <v>2922</v>
-      </c>
-      <c r="G33" s="3" t="s">
-        <v>10</v>
+      <c r="F33" s="4">
+        <v>0</v>
+      </c>
+      <c r="G33" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
@@ -2898,22 +2898,22 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C34" t="s">
         <v>8</v>
       </c>
       <c r="D34" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E34">
         <v>50</v>
       </c>
-      <c r="F34" s="2">
-        <v>263</v>
-      </c>
-      <c r="G34" s="3" t="s">
-        <v>10</v>
+      <c r="F34" s="4">
+        <v>0</v>
+      </c>
+      <c r="G34" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
@@ -2921,22 +2921,22 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C35" t="s">
         <v>8</v>
       </c>
       <c r="D35" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E35">
         <v>50</v>
       </c>
-      <c r="F35" s="2">
-        <v>518</v>
-      </c>
-      <c r="G35" s="3" t="s">
-        <v>10</v>
+      <c r="F35" s="4">
+        <v>0</v>
+      </c>
+      <c r="G35" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
@@ -2944,22 +2944,22 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C36" t="s">
         <v>8</v>
       </c>
       <c r="D36" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E36">
         <v>50</v>
       </c>
-      <c r="F36" s="2">
-        <v>873</v>
-      </c>
-      <c r="G36" s="3" t="s">
-        <v>10</v>
+      <c r="F36" s="4">
+        <v>0</v>
+      </c>
+      <c r="G36" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
@@ -2967,22 +2967,22 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
+        <v>90</v>
+      </c>
+      <c r="C37" t="s">
         <v>91</v>
       </c>
-      <c r="C37" t="s">
+      <c r="D37" t="s">
         <v>92</v>
-      </c>
-      <c r="D37" t="s">
-        <v>93</v>
       </c>
       <c r="E37">
         <v>48</v>
       </c>
-      <c r="F37" s="2">
-        <v>7641</v>
-      </c>
-      <c r="G37" s="3" t="s">
-        <v>10</v>
+      <c r="F37" s="4">
+        <v>0</v>
+      </c>
+      <c r="G37" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
@@ -2990,22 +2990,22 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
+        <v>93</v>
+      </c>
+      <c r="C38" t="s">
         <v>94</v>
       </c>
-      <c r="C38" t="s">
+      <c r="D38" t="s">
         <v>95</v>
-      </c>
-      <c r="D38" t="s">
-        <v>96</v>
       </c>
       <c r="E38">
         <v>48</v>
       </c>
-      <c r="F38" s="2">
-        <v>1483</v>
-      </c>
-      <c r="G38" s="3" t="s">
-        <v>10</v>
+      <c r="F38" s="4">
+        <v>0</v>
+      </c>
+      <c r="G38" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
@@ -3013,22 +3013,22 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
+        <v>96</v>
+      </c>
+      <c r="C39" t="s">
         <v>97</v>
       </c>
-      <c r="C39" t="s">
+      <c r="D39" t="s">
         <v>98</v>
-      </c>
-      <c r="D39" t="s">
-        <v>99</v>
       </c>
       <c r="E39">
         <v>48</v>
       </c>
-      <c r="F39" s="6">
-        <v>0</v>
-      </c>
-      <c r="G39" s="7" t="s">
-        <v>23</v>
+      <c r="F39" s="4">
+        <v>0</v>
+      </c>
+      <c r="G39" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
@@ -3036,22 +3036,22 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
+        <v>99</v>
+      </c>
+      <c r="C40" t="s">
         <v>100</v>
       </c>
-      <c r="C40" t="s">
+      <c r="D40" t="s">
         <v>101</v>
-      </c>
-      <c r="D40" t="s">
-        <v>102</v>
       </c>
       <c r="E40">
         <v>48</v>
       </c>
-      <c r="F40" s="6">
-        <v>0</v>
-      </c>
-      <c r="G40" s="7" t="s">
-        <v>23</v>
+      <c r="F40" s="4">
+        <v>0</v>
+      </c>
+      <c r="G40" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
@@ -3059,22 +3059,22 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
+        <v>102</v>
+      </c>
+      <c r="C41" t="s">
         <v>103</v>
       </c>
-      <c r="C41" t="s">
+      <c r="D41" t="s">
         <v>104</v>
-      </c>
-      <c r="D41" t="s">
-        <v>105</v>
       </c>
       <c r="E41">
         <v>48</v>
       </c>
       <c r="F41" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G41" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
@@ -3082,22 +3082,22 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
+        <v>105</v>
+      </c>
+      <c r="C42" t="s">
         <v>106</v>
       </c>
-      <c r="C42" t="s">
+      <c r="D42" t="s">
         <v>107</v>
-      </c>
-      <c r="D42" t="s">
-        <v>108</v>
       </c>
       <c r="E42">
         <v>48</v>
       </c>
       <c r="F42" s="4">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
@@ -3105,22 +3105,22 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
+        <v>108</v>
+      </c>
+      <c r="C43" t="s">
         <v>109</v>
       </c>
-      <c r="C43" t="s">
+      <c r="D43" t="s">
         <v>110</v>
-      </c>
-      <c r="D43" t="s">
-        <v>111</v>
       </c>
       <c r="E43">
         <v>48</v>
       </c>
-      <c r="F43" s="6">
-        <v>0</v>
-      </c>
-      <c r="G43" s="7" t="s">
-        <v>23</v>
+      <c r="F43" s="4">
+        <v>0</v>
+      </c>
+      <c r="G43" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
@@ -3128,22 +3128,22 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
+        <v>111</v>
+      </c>
+      <c r="C44" t="s">
         <v>112</v>
       </c>
-      <c r="C44" t="s">
+      <c r="D44" t="s">
         <v>113</v>
-      </c>
-      <c r="D44" t="s">
-        <v>114</v>
       </c>
       <c r="E44">
         <v>48</v>
       </c>
-      <c r="F44" s="2">
-        <v>6524</v>
-      </c>
-      <c r="G44" s="3" t="s">
-        <v>10</v>
+      <c r="F44" s="4">
+        <v>0</v>
+      </c>
+      <c r="G44" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
@@ -3151,22 +3151,22 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
+        <v>114</v>
+      </c>
+      <c r="C45" t="s">
         <v>115</v>
       </c>
-      <c r="C45" t="s">
+      <c r="D45" t="s">
         <v>116</v>
-      </c>
-      <c r="D45" t="s">
-        <v>117</v>
       </c>
       <c r="E45">
         <v>48</v>
       </c>
-      <c r="F45" s="6">
-        <v>0</v>
-      </c>
-      <c r="G45" s="7" t="s">
-        <v>23</v>
+      <c r="F45" s="4">
+        <v>0</v>
+      </c>
+      <c r="G45" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
@@ -3174,22 +3174,22 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
+        <v>117</v>
+      </c>
+      <c r="C46" t="s">
         <v>118</v>
       </c>
-      <c r="C46" t="s">
+      <c r="D46" t="s">
         <v>119</v>
-      </c>
-      <c r="D46" t="s">
-        <v>120</v>
       </c>
       <c r="E46">
         <v>48</v>
       </c>
-      <c r="F46" s="6">
-        <v>0</v>
-      </c>
-      <c r="G46" s="7" t="s">
-        <v>23</v>
+      <c r="F46" s="4">
+        <v>0</v>
+      </c>
+      <c r="G46" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
@@ -3197,22 +3197,22 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
+        <v>120</v>
+      </c>
+      <c r="C47" t="s">
         <v>121</v>
       </c>
-      <c r="C47" t="s">
+      <c r="D47" t="s">
         <v>122</v>
-      </c>
-      <c r="D47" t="s">
-        <v>123</v>
       </c>
       <c r="E47">
         <v>48</v>
       </c>
-      <c r="F47" s="2">
-        <v>11965</v>
-      </c>
-      <c r="G47" s="3" t="s">
-        <v>10</v>
+      <c r="F47" s="4">
+        <v>0</v>
+      </c>
+      <c r="G47" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
@@ -3220,22 +3220,22 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
+        <v>123</v>
+      </c>
+      <c r="C48" t="s">
         <v>124</v>
       </c>
-      <c r="C48" t="s">
+      <c r="D48" t="s">
         <v>125</v>
-      </c>
-      <c r="D48" t="s">
-        <v>126</v>
       </c>
       <c r="E48">
         <v>48</v>
       </c>
-      <c r="F48" s="6">
-        <v>0</v>
-      </c>
-      <c r="G48" s="7" t="s">
-        <v>23</v>
+      <c r="F48" s="4">
+        <v>0</v>
+      </c>
+      <c r="G48" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
@@ -3243,22 +3243,22 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
+        <v>126</v>
+      </c>
+      <c r="C49" t="s">
         <v>127</v>
       </c>
-      <c r="C49" t="s">
+      <c r="D49" t="s">
         <v>128</v>
-      </c>
-      <c r="D49" t="s">
-        <v>129</v>
       </c>
       <c r="E49">
         <v>48</v>
       </c>
       <c r="F49" s="4">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G49" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
@@ -3266,22 +3266,22 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
+        <v>129</v>
+      </c>
+      <c r="C50" t="s">
         <v>130</v>
       </c>
-      <c r="C50" t="s">
+      <c r="D50" t="s">
         <v>131</v>
-      </c>
-      <c r="D50" t="s">
-        <v>132</v>
       </c>
       <c r="E50">
         <v>48</v>
       </c>
-      <c r="F50" s="2">
-        <v>5578</v>
-      </c>
-      <c r="G50" s="3" t="s">
-        <v>10</v>
+      <c r="F50" s="4">
+        <v>0</v>
+      </c>
+      <c r="G50" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
@@ -3289,22 +3289,22 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
+        <v>132</v>
+      </c>
+      <c r="C51" t="s">
         <v>133</v>
       </c>
-      <c r="C51" t="s">
+      <c r="D51" t="s">
         <v>134</v>
-      </c>
-      <c r="D51" t="s">
-        <v>135</v>
       </c>
       <c r="E51">
         <v>48</v>
       </c>
-      <c r="F51" s="6">
-        <v>0</v>
-      </c>
-      <c r="G51" s="7" t="s">
-        <v>23</v>
+      <c r="F51" s="4">
+        <v>0</v>
+      </c>
+      <c r="G51" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
@@ -3312,22 +3312,22 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
+        <v>135</v>
+      </c>
+      <c r="C52" t="s">
         <v>136</v>
       </c>
-      <c r="C52" t="s">
+      <c r="D52" t="s">
         <v>137</v>
-      </c>
-      <c r="D52" t="s">
-        <v>138</v>
       </c>
       <c r="E52">
         <v>48</v>
       </c>
       <c r="F52" s="4">
-        <v>117</v>
+        <v>0</v>
       </c>
       <c r="G52" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
@@ -3335,22 +3335,22 @@
         <v>52</v>
       </c>
       <c r="B53" t="s">
+        <v>138</v>
+      </c>
+      <c r="C53" t="s">
         <v>139</v>
       </c>
-      <c r="C53" t="s">
+      <c r="D53" t="s">
         <v>140</v>
-      </c>
-      <c r="D53" t="s">
-        <v>141</v>
       </c>
       <c r="E53">
         <v>48</v>
       </c>
       <c r="F53" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G53" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
@@ -3358,22 +3358,22 @@
         <v>53</v>
       </c>
       <c r="B54" t="s">
+        <v>141</v>
+      </c>
+      <c r="C54" t="s">
         <v>142</v>
       </c>
-      <c r="C54" t="s">
+      <c r="D54" t="s">
         <v>143</v>
-      </c>
-      <c r="D54" t="s">
-        <v>144</v>
       </c>
       <c r="E54">
         <v>48</v>
       </c>
       <c r="F54" s="4">
-        <v>162</v>
+        <v>0</v>
       </c>
       <c r="G54" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
@@ -3381,22 +3381,22 @@
         <v>54</v>
       </c>
       <c r="B55" t="s">
+        <v>144</v>
+      </c>
+      <c r="C55" t="s">
         <v>145</v>
       </c>
-      <c r="C55" t="s">
+      <c r="D55" t="s">
         <v>146</v>
-      </c>
-      <c r="D55" t="s">
-        <v>147</v>
       </c>
       <c r="E55">
         <v>36</v>
       </c>
-      <c r="F55" s="2">
-        <v>1955</v>
-      </c>
-      <c r="G55" s="3" t="s">
-        <v>10</v>
+      <c r="F55" s="4">
+        <v>0</v>
+      </c>
+      <c r="G55" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
@@ -3404,22 +3404,22 @@
         <v>55</v>
       </c>
       <c r="B56" t="s">
+        <v>147</v>
+      </c>
+      <c r="C56" t="s">
         <v>148</v>
       </c>
-      <c r="C56" t="s">
+      <c r="D56" t="s">
         <v>149</v>
-      </c>
-      <c r="D56" t="s">
-        <v>150</v>
       </c>
       <c r="E56">
         <v>36</v>
       </c>
-      <c r="F56" s="2">
-        <v>196</v>
-      </c>
-      <c r="G56" s="3" t="s">
-        <v>10</v>
+      <c r="F56" s="4">
+        <v>0</v>
+      </c>
+      <c r="G56" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
@@ -3427,22 +3427,22 @@
         <v>56</v>
       </c>
       <c r="B57" t="s">
+        <v>150</v>
+      </c>
+      <c r="C57" t="s">
         <v>151</v>
       </c>
-      <c r="C57" t="s">
+      <c r="D57" t="s">
         <v>152</v>
-      </c>
-      <c r="D57" t="s">
-        <v>153</v>
       </c>
       <c r="E57">
         <v>36</v>
       </c>
-      <c r="F57" s="2">
-        <v>2190</v>
-      </c>
-      <c r="G57" s="3" t="s">
-        <v>10</v>
+      <c r="F57" s="4">
+        <v>0</v>
+      </c>
+      <c r="G57" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
@@ -3450,22 +3450,22 @@
         <v>57</v>
       </c>
       <c r="B58" t="s">
+        <v>153</v>
+      </c>
+      <c r="C58" t="s">
         <v>154</v>
       </c>
-      <c r="C58" t="s">
+      <c r="D58" t="s">
         <v>155</v>
-      </c>
-      <c r="D58" t="s">
-        <v>156</v>
       </c>
       <c r="E58">
         <v>36</v>
       </c>
-      <c r="F58" s="6">
-        <v>0</v>
-      </c>
-      <c r="G58" s="7" t="s">
-        <v>23</v>
+      <c r="F58" s="4">
+        <v>0</v>
+      </c>
+      <c r="G58" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
@@ -3473,22 +3473,22 @@
         <v>58</v>
       </c>
       <c r="B59" t="s">
+        <v>156</v>
+      </c>
+      <c r="C59" t="s">
         <v>157</v>
       </c>
-      <c r="C59" t="s">
+      <c r="D59" t="s">
         <v>158</v>
-      </c>
-      <c r="D59" t="s">
-        <v>159</v>
       </c>
       <c r="E59">
         <v>36</v>
       </c>
-      <c r="F59" s="6">
-        <v>0</v>
-      </c>
-      <c r="G59" s="7" t="s">
-        <v>23</v>
+      <c r="F59" s="4">
+        <v>0</v>
+      </c>
+      <c r="G59" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
@@ -3496,22 +3496,22 @@
         <v>59</v>
       </c>
       <c r="B60" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C60" t="s">
         <v>8</v>
       </c>
       <c r="D60" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E60">
         <v>36</v>
       </c>
-      <c r="F60" s="2">
-        <v>1377</v>
-      </c>
-      <c r="G60" s="3" t="s">
-        <v>10</v>
+      <c r="F60" s="4">
+        <v>0</v>
+      </c>
+      <c r="G60" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
@@ -3519,22 +3519,22 @@
         <v>60</v>
       </c>
       <c r="B61" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C61" t="s">
         <v>8</v>
       </c>
       <c r="D61" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E61">
         <v>36</v>
       </c>
-      <c r="F61" s="6">
-        <v>0</v>
-      </c>
-      <c r="G61" s="7" t="s">
-        <v>23</v>
+      <c r="F61" s="4">
+        <v>0</v>
+      </c>
+      <c r="G61" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
@@ -3542,22 +3542,22 @@
         <v>61</v>
       </c>
       <c r="B62" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C62" t="s">
         <v>8</v>
       </c>
       <c r="D62" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E62">
         <v>36</v>
       </c>
-      <c r="F62" s="2">
-        <v>915</v>
-      </c>
-      <c r="G62" s="3" t="s">
-        <v>10</v>
+      <c r="F62" s="4">
+        <v>0</v>
+      </c>
+      <c r="G62" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
@@ -3565,22 +3565,22 @@
         <v>62</v>
       </c>
       <c r="B63" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C63" t="s">
         <v>8</v>
       </c>
       <c r="D63" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E63">
         <v>36</v>
       </c>
-      <c r="F63" s="2">
-        <v>798</v>
-      </c>
-      <c r="G63" s="3" t="s">
-        <v>10</v>
+      <c r="F63" s="4">
+        <v>0</v>
+      </c>
+      <c r="G63" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
@@ -3588,22 +3588,22 @@
         <v>63</v>
       </c>
       <c r="B64" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C64" t="s">
         <v>8</v>
       </c>
       <c r="D64" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E64">
         <v>48</v>
       </c>
-      <c r="F64" s="2">
-        <v>418</v>
-      </c>
-      <c r="G64" s="3" t="s">
+      <c r="F64" s="6">
         <v>10</v>
+      </c>
+      <c r="G64" s="7" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
@@ -3622,11 +3622,11 @@
       <c r="E65">
         <v>48</v>
       </c>
-      <c r="F65" s="2">
-        <v>1218</v>
-      </c>
-      <c r="G65" s="3" t="s">
-        <v>10</v>
+      <c r="F65" s="4">
+        <v>0</v>
+      </c>
+      <c r="G65" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.25">
@@ -3645,11 +3645,11 @@
       <c r="E66">
         <v>60</v>
       </c>
-      <c r="F66" s="2">
-        <v>5188</v>
-      </c>
-      <c r="G66" s="3" t="s">
-        <v>10</v>
+      <c r="F66" s="4">
+        <v>0</v>
+      </c>
+      <c r="G66" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
@@ -3668,11 +3668,11 @@
       <c r="E67">
         <v>60</v>
       </c>
-      <c r="F67" s="2">
-        <v>1226</v>
-      </c>
-      <c r="G67" s="3" t="s">
-        <v>10</v>
+      <c r="F67" s="4">
+        <v>0</v>
+      </c>
+      <c r="G67" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
@@ -3691,11 +3691,11 @@
       <c r="E68">
         <v>60</v>
       </c>
-      <c r="F68" s="2">
-        <v>2119</v>
-      </c>
-      <c r="G68" s="3" t="s">
-        <v>10</v>
+      <c r="F68" s="4">
+        <v>0</v>
+      </c>
+      <c r="G68" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.25">
@@ -3714,11 +3714,11 @@
       <c r="E69">
         <v>60</v>
       </c>
-      <c r="F69" s="2">
-        <v>1118</v>
-      </c>
-      <c r="G69" s="3" t="s">
-        <v>10</v>
+      <c r="F69" s="4">
+        <v>0</v>
+      </c>
+      <c r="G69" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.25">
@@ -3737,11 +3737,11 @@
       <c r="E70">
         <v>60</v>
       </c>
-      <c r="F70" s="2">
-        <v>4180</v>
-      </c>
-      <c r="G70" s="3" t="s">
-        <v>10</v>
+      <c r="F70" s="4">
+        <v>0</v>
+      </c>
+      <c r="G70" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
@@ -3760,11 +3760,11 @@
       <c r="E71">
         <v>60</v>
       </c>
-      <c r="F71" s="2">
-        <v>5085</v>
-      </c>
-      <c r="G71" s="3" t="s">
-        <v>10</v>
+      <c r="F71" s="4">
+        <v>0</v>
+      </c>
+      <c r="G71" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.25">
@@ -3783,11 +3783,11 @@
       <c r="E72">
         <v>60</v>
       </c>
-      <c r="F72" s="6">
-        <v>0</v>
-      </c>
-      <c r="G72" s="7" t="s">
-        <v>23</v>
+      <c r="F72" s="4">
+        <v>0</v>
+      </c>
+      <c r="G72" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
@@ -3806,11 +3806,11 @@
       <c r="E73">
         <v>60</v>
       </c>
-      <c r="F73" s="2">
-        <v>3198</v>
-      </c>
-      <c r="G73" s="3" t="s">
-        <v>10</v>
+      <c r="F73" s="4">
+        <v>0</v>
+      </c>
+      <c r="G73" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.25">
@@ -3829,11 +3829,11 @@
       <c r="E74">
         <v>60</v>
       </c>
-      <c r="F74" s="2">
-        <v>1302</v>
-      </c>
-      <c r="G74" s="3" t="s">
-        <v>10</v>
+      <c r="F74" s="4">
+        <v>0</v>
+      </c>
+      <c r="G74" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.25">
@@ -3852,11 +3852,11 @@
       <c r="E75">
         <v>60</v>
       </c>
-      <c r="F75" s="2">
-        <v>4399</v>
-      </c>
-      <c r="G75" s="3" t="s">
-        <v>10</v>
+      <c r="F75" s="4">
+        <v>0</v>
+      </c>
+      <c r="G75" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.25">
@@ -3875,11 +3875,11 @@
       <c r="E76">
         <v>60</v>
       </c>
-      <c r="F76" s="2">
-        <v>8596</v>
-      </c>
-      <c r="G76" s="3" t="s">
-        <v>10</v>
+      <c r="F76" s="4">
+        <v>0</v>
+      </c>
+      <c r="G76" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.25">
@@ -3898,11 +3898,11 @@
       <c r="E77">
         <v>60</v>
       </c>
-      <c r="F77" s="2">
-        <v>3977</v>
-      </c>
-      <c r="G77" s="3" t="s">
-        <v>10</v>
+      <c r="F77" s="4">
+        <v>0</v>
+      </c>
+      <c r="G77" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.25">
@@ -3921,11 +3921,11 @@
       <c r="E78">
         <v>60</v>
       </c>
-      <c r="F78" s="2">
-        <v>6465</v>
-      </c>
-      <c r="G78" s="3" t="s">
-        <v>10</v>
+      <c r="F78" s="4">
+        <v>0</v>
+      </c>
+      <c r="G78" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.25">
@@ -3944,11 +3944,11 @@
       <c r="E79">
         <v>60</v>
       </c>
-      <c r="F79" s="2">
-        <v>5202</v>
-      </c>
-      <c r="G79" s="3" t="s">
-        <v>10</v>
+      <c r="F79" s="4">
+        <v>0</v>
+      </c>
+      <c r="G79" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.25">
@@ -3968,10 +3968,10 @@
         <v>60</v>
       </c>
       <c r="F80" s="4">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="G80" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.25">
@@ -3991,10 +3991,10 @@
         <v>60</v>
       </c>
       <c r="F81" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G81" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.25">
@@ -4013,11 +4013,11 @@
       <c r="E82">
         <v>60</v>
       </c>
-      <c r="F82" s="2">
-        <v>1124</v>
-      </c>
-      <c r="G82" s="3" t="s">
-        <v>10</v>
+      <c r="F82" s="4">
+        <v>0</v>
+      </c>
+      <c r="G82" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.25">
@@ -4036,11 +4036,11 @@
       <c r="E83">
         <v>60</v>
       </c>
-      <c r="F83" s="2">
-        <v>1037</v>
-      </c>
-      <c r="G83" s="3" t="s">
-        <v>10</v>
+      <c r="F83" s="4">
+        <v>0</v>
+      </c>
+      <c r="G83" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.25">
@@ -4059,11 +4059,11 @@
       <c r="E84">
         <v>60</v>
       </c>
-      <c r="F84" s="6">
-        <v>0</v>
-      </c>
-      <c r="G84" s="7" t="s">
-        <v>23</v>
+      <c r="F84" s="4">
+        <v>0</v>
+      </c>
+      <c r="G84" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.25">
@@ -4083,10 +4083,10 @@
         <v>60</v>
       </c>
       <c r="F85" s="4">
-        <v>154</v>
+        <v>0</v>
       </c>
       <c r="G85" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.25">
@@ -4105,11 +4105,11 @@
       <c r="E86">
         <v>60</v>
       </c>
-      <c r="F86" s="2">
-        <v>333</v>
-      </c>
-      <c r="G86" s="3" t="s">
-        <v>10</v>
+      <c r="F86" s="4">
+        <v>0</v>
+      </c>
+      <c r="G86" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.25">
@@ -4128,11 +4128,11 @@
       <c r="E87">
         <v>60</v>
       </c>
-      <c r="F87" s="2">
-        <v>1531</v>
-      </c>
-      <c r="G87" s="3" t="s">
-        <v>10</v>
+      <c r="F87" s="4">
+        <v>0</v>
+      </c>
+      <c r="G87" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.25">
@@ -4151,11 +4151,11 @@
       <c r="E88">
         <v>60</v>
       </c>
-      <c r="F88" s="6">
-        <v>0</v>
-      </c>
-      <c r="G88" s="7" t="s">
-        <v>23</v>
+      <c r="F88" s="4">
+        <v>0</v>
+      </c>
+      <c r="G88" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.25">
@@ -4174,11 +4174,11 @@
       <c r="E89">
         <v>60</v>
       </c>
-      <c r="F89" s="6">
-        <v>0</v>
-      </c>
-      <c r="G89" s="7" t="s">
-        <v>23</v>
+      <c r="F89" s="4">
+        <v>0</v>
+      </c>
+      <c r="G89" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.25">
@@ -4197,11 +4197,11 @@
       <c r="E90">
         <v>60</v>
       </c>
-      <c r="F90" s="2">
-        <v>734</v>
-      </c>
-      <c r="G90" s="3" t="s">
-        <v>10</v>
+      <c r="F90" s="4">
+        <v>0</v>
+      </c>
+      <c r="G90" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.25">
@@ -4220,11 +4220,11 @@
       <c r="E91">
         <v>60</v>
       </c>
-      <c r="F91" s="2">
-        <v>1518</v>
-      </c>
-      <c r="G91" s="3" t="s">
-        <v>10</v>
+      <c r="F91" s="4">
+        <v>0</v>
+      </c>
+      <c r="G91" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.25">
@@ -4243,11 +4243,11 @@
       <c r="E92">
         <v>60</v>
       </c>
-      <c r="F92" s="2">
-        <v>1372</v>
-      </c>
-      <c r="G92" s="3" t="s">
-        <v>10</v>
+      <c r="F92" s="4">
+        <v>0</v>
+      </c>
+      <c r="G92" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.25">
@@ -4266,11 +4266,11 @@
       <c r="E93">
         <v>60</v>
       </c>
-      <c r="F93" s="2">
-        <v>1251</v>
-      </c>
-      <c r="G93" s="3" t="s">
-        <v>10</v>
+      <c r="F93" s="4">
+        <v>0</v>
+      </c>
+      <c r="G93" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.25">
@@ -4289,11 +4289,11 @@
       <c r="E94">
         <v>60</v>
       </c>
-      <c r="F94" s="2">
-        <v>1399</v>
-      </c>
-      <c r="G94" s="3" t="s">
-        <v>10</v>
+      <c r="F94" s="4">
+        <v>0</v>
+      </c>
+      <c r="G94" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.25">
@@ -4312,11 +4312,11 @@
       <c r="E95">
         <v>60</v>
       </c>
-      <c r="F95" s="6">
-        <v>0</v>
-      </c>
-      <c r="G95" s="7" t="s">
-        <v>23</v>
+      <c r="F95" s="4">
+        <v>0</v>
+      </c>
+      <c r="G95" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.25">
@@ -4335,11 +4335,11 @@
       <c r="E96">
         <v>60</v>
       </c>
-      <c r="F96" s="2">
-        <v>2485</v>
-      </c>
-      <c r="G96" s="3" t="s">
-        <v>10</v>
+      <c r="F96" s="4">
+        <v>0</v>
+      </c>
+      <c r="G96" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.25">
@@ -4358,11 +4358,11 @@
       <c r="E97">
         <v>60</v>
       </c>
-      <c r="F97" s="2">
-        <v>5025</v>
-      </c>
-      <c r="G97" s="3" t="s">
-        <v>10</v>
+      <c r="F97" s="4">
+        <v>0</v>
+      </c>
+      <c r="G97" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.25">
@@ -4381,11 +4381,11 @@
       <c r="E98">
         <v>60</v>
       </c>
-      <c r="F98" s="2">
-        <v>3434</v>
-      </c>
-      <c r="G98" s="3" t="s">
-        <v>10</v>
+      <c r="F98" s="4">
+        <v>0</v>
+      </c>
+      <c r="G98" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.25">
@@ -4404,11 +4404,11 @@
       <c r="E99">
         <v>60</v>
       </c>
-      <c r="F99" s="2">
-        <v>3915</v>
-      </c>
-      <c r="G99" s="3" t="s">
-        <v>10</v>
+      <c r="F99" s="4">
+        <v>0</v>
+      </c>
+      <c r="G99" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.25">
@@ -4427,11 +4427,11 @@
       <c r="E100">
         <v>60</v>
       </c>
-      <c r="F100" s="2">
-        <v>1544</v>
-      </c>
-      <c r="G100" s="3" t="s">
-        <v>10</v>
+      <c r="F100" s="4">
+        <v>0</v>
+      </c>
+      <c r="G100" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.25">
@@ -4450,11 +4450,11 @@
       <c r="E101">
         <v>60</v>
       </c>
-      <c r="F101" s="2">
-        <v>5802</v>
-      </c>
-      <c r="G101" s="3" t="s">
-        <v>10</v>
+      <c r="F101" s="4">
+        <v>0</v>
+      </c>
+      <c r="G101" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.25">
@@ -4473,11 +4473,11 @@
       <c r="E102">
         <v>60</v>
       </c>
-      <c r="F102" s="2">
-        <v>3253</v>
-      </c>
-      <c r="G102" s="3" t="s">
-        <v>10</v>
+      <c r="F102" s="4">
+        <v>0</v>
+      </c>
+      <c r="G102" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.25">
@@ -4496,11 +4496,11 @@
       <c r="E103">
         <v>60</v>
       </c>
-      <c r="F103" s="2">
-        <v>1816</v>
-      </c>
-      <c r="G103" s="3" t="s">
-        <v>10</v>
+      <c r="F103" s="4">
+        <v>0</v>
+      </c>
+      <c r="G103" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.25">
@@ -4519,11 +4519,11 @@
       <c r="E104">
         <v>60</v>
       </c>
-      <c r="F104" s="2">
-        <v>368</v>
-      </c>
-      <c r="G104" s="3" t="s">
-        <v>10</v>
+      <c r="F104" s="4">
+        <v>0</v>
+      </c>
+      <c r="G104" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.25">
@@ -4542,11 +4542,11 @@
       <c r="E105">
         <v>60</v>
       </c>
-      <c r="F105" s="6">
-        <v>0</v>
-      </c>
-      <c r="G105" s="7" t="s">
-        <v>23</v>
+      <c r="F105" s="4">
+        <v>0</v>
+      </c>
+      <c r="G105" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.25">
@@ -4565,11 +4565,11 @@
       <c r="E106">
         <v>60</v>
       </c>
-      <c r="F106" s="2">
-        <v>852</v>
-      </c>
-      <c r="G106" s="3" t="s">
-        <v>10</v>
+      <c r="F106" s="4">
+        <v>0</v>
+      </c>
+      <c r="G106" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.25">
@@ -4588,11 +4588,11 @@
       <c r="E107">
         <v>60</v>
       </c>
-      <c r="F107" s="2">
-        <v>5594</v>
-      </c>
-      <c r="G107" s="3" t="s">
-        <v>10</v>
+      <c r="F107" s="4">
+        <v>0</v>
+      </c>
+      <c r="G107" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.25">
@@ -4611,11 +4611,11 @@
       <c r="E108">
         <v>60</v>
       </c>
-      <c r="F108" s="2">
-        <v>1998</v>
-      </c>
-      <c r="G108" s="3" t="s">
-        <v>10</v>
+      <c r="F108" s="4">
+        <v>0</v>
+      </c>
+      <c r="G108" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.25">
@@ -4634,11 +4634,11 @@
       <c r="E109">
         <v>60</v>
       </c>
-      <c r="F109" s="2">
-        <v>1725</v>
-      </c>
-      <c r="G109" s="3" t="s">
-        <v>10</v>
+      <c r="F109" s="4">
+        <v>0</v>
+      </c>
+      <c r="G109" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.25">
@@ -4657,11 +4657,11 @@
       <c r="E110">
         <v>60</v>
       </c>
-      <c r="F110" s="2">
-        <v>1887</v>
-      </c>
-      <c r="G110" s="3" t="s">
-        <v>10</v>
+      <c r="F110" s="4">
+        <v>0</v>
+      </c>
+      <c r="G110" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.25">
@@ -4680,11 +4680,11 @@
       <c r="E111">
         <v>60</v>
       </c>
-      <c r="F111" s="2">
-        <v>6130</v>
-      </c>
-      <c r="G111" s="3" t="s">
-        <v>10</v>
+      <c r="F111" s="4">
+        <v>0</v>
+      </c>
+      <c r="G111" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.25">
@@ -4703,11 +4703,11 @@
       <c r="E112">
         <v>60</v>
       </c>
-      <c r="F112" s="2">
-        <v>7112</v>
-      </c>
-      <c r="G112" s="3" t="s">
-        <v>10</v>
+      <c r="F112" s="4">
+        <v>0</v>
+      </c>
+      <c r="G112" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.25">
@@ -4726,11 +4726,11 @@
       <c r="E113">
         <v>60</v>
       </c>
-      <c r="F113" s="2">
-        <v>6610</v>
-      </c>
-      <c r="G113" s="3" t="s">
-        <v>10</v>
+      <c r="F113" s="4">
+        <v>0</v>
+      </c>
+      <c r="G113" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.25">
@@ -4749,11 +4749,11 @@
       <c r="E114">
         <v>60</v>
       </c>
-      <c r="F114" s="2">
-        <v>11151</v>
-      </c>
-      <c r="G114" s="3" t="s">
-        <v>10</v>
+      <c r="F114" s="4">
+        <v>0</v>
+      </c>
+      <c r="G114" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.25">
@@ -4772,11 +4772,11 @@
       <c r="E115">
         <v>1</v>
       </c>
-      <c r="F115" s="2">
-        <v>239</v>
-      </c>
-      <c r="G115" s="3" t="s">
-        <v>10</v>
+      <c r="F115" s="4">
+        <v>0</v>
+      </c>
+      <c r="G115" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.25">
@@ -4795,11 +4795,11 @@
       <c r="E116">
         <v>1</v>
       </c>
-      <c r="F116" s="2">
-        <v>85</v>
-      </c>
-      <c r="G116" s="3" t="s">
-        <v>10</v>
+      <c r="F116" s="4">
+        <v>0</v>
+      </c>
+      <c r="G116" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.25">
@@ -4818,11 +4818,11 @@
       <c r="E117">
         <v>1</v>
       </c>
-      <c r="F117" s="2">
-        <v>273</v>
-      </c>
-      <c r="G117" s="3" t="s">
-        <v>10</v>
+      <c r="F117" s="4">
+        <v>0</v>
+      </c>
+      <c r="G117" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="118" spans="1:7" x14ac:dyDescent="0.25">
@@ -4841,11 +4841,11 @@
       <c r="E118">
         <v>1</v>
       </c>
-      <c r="F118" s="2">
-        <v>272</v>
-      </c>
-      <c r="G118" s="3" t="s">
-        <v>10</v>
+      <c r="F118" s="4">
+        <v>0</v>
+      </c>
+      <c r="G118" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="119" spans="1:7" x14ac:dyDescent="0.25">
@@ -4864,11 +4864,11 @@
       <c r="E119">
         <v>12</v>
       </c>
-      <c r="F119" s="6">
-        <v>0</v>
-      </c>
-      <c r="G119" s="7" t="s">
-        <v>23</v>
+      <c r="F119" s="4">
+        <v>0</v>
+      </c>
+      <c r="G119" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="120" spans="1:7" x14ac:dyDescent="0.25">
@@ -4887,11 +4887,11 @@
       <c r="E120">
         <v>36</v>
       </c>
-      <c r="F120" s="2">
-        <v>261</v>
-      </c>
-      <c r="G120" s="3" t="s">
-        <v>10</v>
+      <c r="F120" s="4">
+        <v>0</v>
+      </c>
+      <c r="G120" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.25">
@@ -4910,11 +4910,11 @@
       <c r="E121">
         <v>36</v>
       </c>
-      <c r="F121" s="6">
-        <v>0</v>
-      </c>
-      <c r="G121" s="7" t="s">
-        <v>23</v>
+      <c r="F121" s="4">
+        <v>0</v>
+      </c>
+      <c r="G121" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="122" spans="1:7" x14ac:dyDescent="0.25">
@@ -4933,11 +4933,11 @@
       <c r="E122">
         <v>12</v>
       </c>
-      <c r="F122" s="2">
-        <v>2925</v>
-      </c>
-      <c r="G122" s="3" t="s">
-        <v>10</v>
+      <c r="F122" s="4">
+        <v>0</v>
+      </c>
+      <c r="G122" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="123" spans="1:7" x14ac:dyDescent="0.25">
@@ -4957,10 +4957,10 @@
         <v>36</v>
       </c>
       <c r="F123" s="4">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G123" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="124" spans="1:7" x14ac:dyDescent="0.25">
@@ -4979,11 +4979,11 @@
       <c r="E124">
         <v>12</v>
       </c>
-      <c r="F124" s="2">
-        <v>2515</v>
-      </c>
-      <c r="G124" s="3" t="s">
-        <v>10</v>
+      <c r="F124" s="4">
+        <v>0</v>
+      </c>
+      <c r="G124" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="125" spans="1:7" x14ac:dyDescent="0.25">
@@ -5002,11 +5002,11 @@
       <c r="E125">
         <v>36</v>
       </c>
-      <c r="F125" s="2">
-        <v>969</v>
-      </c>
-      <c r="G125" s="3" t="s">
-        <v>10</v>
+      <c r="F125" s="4">
+        <v>0</v>
+      </c>
+      <c r="G125" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="126" spans="1:7" x14ac:dyDescent="0.25">
@@ -5025,11 +5025,11 @@
       <c r="E126">
         <v>120</v>
       </c>
-      <c r="F126" s="2">
-        <v>2200</v>
-      </c>
-      <c r="G126" s="3" t="s">
-        <v>10</v>
+      <c r="F126" s="4">
+        <v>0</v>
+      </c>
+      <c r="G126" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="127" spans="1:7" x14ac:dyDescent="0.25">
@@ -5049,10 +5049,10 @@
         <v>120</v>
       </c>
       <c r="F127" s="4">
-        <v>155</v>
+        <v>0</v>
       </c>
       <c r="G127" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="128" spans="1:7" x14ac:dyDescent="0.25">
@@ -5072,10 +5072,10 @@
         <v>120</v>
       </c>
       <c r="F128" s="4">
-        <v>519</v>
+        <v>0</v>
       </c>
       <c r="G128" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="129" spans="1:7" x14ac:dyDescent="0.25">
@@ -5094,11 +5094,11 @@
       <c r="E129">
         <v>120</v>
       </c>
-      <c r="F129" s="2">
-        <v>1067</v>
-      </c>
-      <c r="G129" s="3" t="s">
-        <v>10</v>
+      <c r="F129" s="4">
+        <v>0</v>
+      </c>
+      <c r="G129" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="130" spans="1:7" x14ac:dyDescent="0.25">
@@ -5117,11 +5117,11 @@
       <c r="E130">
         <v>120</v>
       </c>
-      <c r="F130" s="2">
-        <v>884</v>
-      </c>
-      <c r="G130" s="3" t="s">
-        <v>10</v>
+      <c r="F130" s="4">
+        <v>0</v>
+      </c>
+      <c r="G130" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="131" spans="1:7" x14ac:dyDescent="0.25">
@@ -5141,10 +5141,10 @@
         <v>120</v>
       </c>
       <c r="F131" s="4">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="G131" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="132" spans="1:7" x14ac:dyDescent="0.25">
@@ -5164,10 +5164,10 @@
         <v>120</v>
       </c>
       <c r="F132" s="4">
-        <v>233</v>
+        <v>0</v>
       </c>
       <c r="G132" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="133" spans="1:7" x14ac:dyDescent="0.25">
@@ -5186,11 +5186,11 @@
       <c r="E133">
         <v>120</v>
       </c>
-      <c r="F133" s="2">
-        <v>6592</v>
-      </c>
-      <c r="G133" s="3" t="s">
-        <v>10</v>
+      <c r="F133" s="4">
+        <v>0</v>
+      </c>
+      <c r="G133" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="134" spans="1:7" x14ac:dyDescent="0.25">
@@ -5209,11 +5209,11 @@
       <c r="E134">
         <v>120</v>
       </c>
-      <c r="F134" s="2">
-        <v>1017</v>
-      </c>
-      <c r="G134" s="3" t="s">
-        <v>10</v>
+      <c r="F134" s="4">
+        <v>0</v>
+      </c>
+      <c r="G134" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="135" spans="1:7" x14ac:dyDescent="0.25">
@@ -5233,10 +5233,10 @@
         <v>120</v>
       </c>
       <c r="F135" s="4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G135" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="136" spans="1:7" x14ac:dyDescent="0.25">
@@ -5255,11 +5255,11 @@
       <c r="E136">
         <v>120</v>
       </c>
-      <c r="F136" s="2">
-        <v>4015</v>
-      </c>
-      <c r="G136" s="3" t="s">
-        <v>10</v>
+      <c r="F136" s="4">
+        <v>0</v>
+      </c>
+      <c r="G136" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="137" spans="1:7" x14ac:dyDescent="0.25">
@@ -5278,11 +5278,11 @@
       <c r="E137">
         <v>120</v>
       </c>
-      <c r="F137" s="2">
-        <v>1904</v>
-      </c>
-      <c r="G137" s="3" t="s">
-        <v>10</v>
+      <c r="F137" s="4">
+        <v>0</v>
+      </c>
+      <c r="G137" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="138" spans="1:7" x14ac:dyDescent="0.25">
@@ -5302,10 +5302,10 @@
         <v>120</v>
       </c>
       <c r="F138" s="4">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G138" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="139" spans="1:7" x14ac:dyDescent="0.25">
@@ -5324,11 +5324,11 @@
       <c r="E139">
         <v>120</v>
       </c>
-      <c r="F139" s="2">
-        <v>4463</v>
-      </c>
-      <c r="G139" s="3" t="s">
-        <v>10</v>
+      <c r="F139" s="4">
+        <v>0</v>
+      </c>
+      <c r="G139" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="140" spans="1:7" x14ac:dyDescent="0.25">
@@ -5348,10 +5348,10 @@
         <v>120</v>
       </c>
       <c r="F140" s="4">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G140" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="141" spans="1:7" x14ac:dyDescent="0.25">
@@ -5370,11 +5370,11 @@
       <c r="E141">
         <v>120</v>
       </c>
-      <c r="F141" s="2">
-        <v>4217</v>
-      </c>
-      <c r="G141" s="3" t="s">
-        <v>10</v>
+      <c r="F141" s="4">
+        <v>0</v>
+      </c>
+      <c r="G141" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="142" spans="1:7" x14ac:dyDescent="0.25">
@@ -5393,11 +5393,11 @@
       <c r="E142">
         <v>120</v>
       </c>
-      <c r="F142" s="2">
-        <v>3364</v>
-      </c>
-      <c r="G142" s="3" t="s">
-        <v>10</v>
+      <c r="F142" s="4">
+        <v>0</v>
+      </c>
+      <c r="G142" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="143" spans="1:7" x14ac:dyDescent="0.25">
@@ -5417,10 +5417,10 @@
         <v>120</v>
       </c>
       <c r="F143" s="4">
-        <v>514</v>
+        <v>0</v>
       </c>
       <c r="G143" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="144" spans="1:7" x14ac:dyDescent="0.25">
@@ -5439,11 +5439,11 @@
       <c r="E144">
         <v>120</v>
       </c>
-      <c r="F144" s="6">
-        <v>0</v>
-      </c>
-      <c r="G144" s="7" t="s">
-        <v>23</v>
+      <c r="F144" s="4">
+        <v>0</v>
+      </c>
+      <c r="G144" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="145" spans="1:7" x14ac:dyDescent="0.25">
@@ -5463,10 +5463,10 @@
         <v>120</v>
       </c>
       <c r="F145" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G145" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="146" spans="1:7" x14ac:dyDescent="0.25">
@@ -5485,11 +5485,11 @@
       <c r="E146">
         <v>60</v>
       </c>
-      <c r="F146" s="2">
-        <v>752</v>
-      </c>
-      <c r="G146" s="3" t="s">
-        <v>10</v>
+      <c r="F146" s="4">
+        <v>0</v>
+      </c>
+      <c r="G146" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="147" spans="1:7" x14ac:dyDescent="0.25">
@@ -5508,11 +5508,11 @@
       <c r="E147">
         <v>120</v>
       </c>
-      <c r="F147" s="2">
-        <v>1964</v>
-      </c>
-      <c r="G147" s="3" t="s">
-        <v>10</v>
+      <c r="F147" s="4">
+        <v>0</v>
+      </c>
+      <c r="G147" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="148" spans="1:7" x14ac:dyDescent="0.25">
@@ -5532,10 +5532,10 @@
         <v>120</v>
       </c>
       <c r="F148" s="4">
-        <v>397</v>
+        <v>0</v>
       </c>
       <c r="G148" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="149" spans="1:7" x14ac:dyDescent="0.25">
@@ -5555,10 +5555,10 @@
         <v>120</v>
       </c>
       <c r="F149" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G149" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="150" spans="1:7" x14ac:dyDescent="0.25">
@@ -5578,10 +5578,10 @@
         <v>120</v>
       </c>
       <c r="F150" s="4">
-        <v>386</v>
+        <v>0</v>
       </c>
       <c r="G150" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="151" spans="1:7" x14ac:dyDescent="0.25">
@@ -5600,11 +5600,11 @@
       <c r="E151">
         <v>120</v>
       </c>
-      <c r="F151" s="2">
-        <v>2007</v>
-      </c>
-      <c r="G151" s="3" t="s">
-        <v>10</v>
+      <c r="F151" s="4">
+        <v>0</v>
+      </c>
+      <c r="G151" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="152" spans="1:7" x14ac:dyDescent="0.25">
@@ -5624,10 +5624,10 @@
         <v>120</v>
       </c>
       <c r="F152" s="4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G152" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="153" spans="1:7" x14ac:dyDescent="0.25">
@@ -5646,11 +5646,11 @@
       <c r="E153">
         <v>120</v>
       </c>
-      <c r="F153" s="6">
-        <v>0</v>
-      </c>
-      <c r="G153" s="7" t="s">
-        <v>23</v>
+      <c r="F153" s="4">
+        <v>0</v>
+      </c>
+      <c r="G153" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="154" spans="1:7" x14ac:dyDescent="0.25">
@@ -5669,11 +5669,11 @@
       <c r="E154">
         <v>120</v>
       </c>
-      <c r="F154" s="2">
-        <v>3277</v>
-      </c>
-      <c r="G154" s="3" t="s">
-        <v>10</v>
+      <c r="F154" s="4">
+        <v>0</v>
+      </c>
+      <c r="G154" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="155" spans="1:7" x14ac:dyDescent="0.25">
@@ -5692,11 +5692,11 @@
       <c r="E155">
         <v>120</v>
       </c>
-      <c r="F155" s="2">
-        <v>908</v>
-      </c>
-      <c r="G155" s="3" t="s">
-        <v>10</v>
+      <c r="F155" s="4">
+        <v>0</v>
+      </c>
+      <c r="G155" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="156" spans="1:7" x14ac:dyDescent="0.25">
@@ -5716,10 +5716,10 @@
         <v>120</v>
       </c>
       <c r="F156" s="4">
-        <v>306</v>
+        <v>0</v>
       </c>
       <c r="G156" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="157" spans="1:7" x14ac:dyDescent="0.25">
@@ -5738,11 +5738,11 @@
       <c r="E157">
         <v>120</v>
       </c>
-      <c r="F157" s="2">
-        <v>3114</v>
-      </c>
-      <c r="G157" s="3" t="s">
-        <v>10</v>
+      <c r="F157" s="4">
+        <v>0</v>
+      </c>
+      <c r="G157" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="158" spans="1:7" x14ac:dyDescent="0.25">
@@ -5761,11 +5761,11 @@
       <c r="E158">
         <v>120</v>
       </c>
-      <c r="F158" s="2">
-        <v>1101</v>
-      </c>
-      <c r="G158" s="3" t="s">
-        <v>10</v>
+      <c r="F158" s="4">
+        <v>0</v>
+      </c>
+      <c r="G158" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="159" spans="1:7" x14ac:dyDescent="0.25">
@@ -5784,11 +5784,11 @@
       <c r="E159">
         <v>120</v>
       </c>
-      <c r="F159" s="2">
-        <v>3978</v>
-      </c>
-      <c r="G159" s="3" t="s">
-        <v>10</v>
+      <c r="F159" s="4">
+        <v>0</v>
+      </c>
+      <c r="G159" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="160" spans="1:7" x14ac:dyDescent="0.25">
@@ -5808,10 +5808,10 @@
         <v>120</v>
       </c>
       <c r="F160" s="4">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G160" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="161" spans="1:7" x14ac:dyDescent="0.25">
@@ -5830,11 +5830,11 @@
       <c r="E161">
         <v>120</v>
       </c>
-      <c r="F161" s="2">
-        <v>1926</v>
-      </c>
-      <c r="G161" s="3" t="s">
-        <v>10</v>
+      <c r="F161" s="4">
+        <v>0</v>
+      </c>
+      <c r="G161" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="162" spans="1:7" x14ac:dyDescent="0.25">
@@ -5853,11 +5853,11 @@
       <c r="E162">
         <v>120</v>
       </c>
-      <c r="F162" s="2">
-        <v>4672</v>
-      </c>
-      <c r="G162" s="3" t="s">
-        <v>10</v>
+      <c r="F162" s="4">
+        <v>0</v>
+      </c>
+      <c r="G162" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="163" spans="1:7" x14ac:dyDescent="0.25">
@@ -5876,11 +5876,11 @@
       <c r="E163">
         <v>120</v>
       </c>
-      <c r="F163" s="2">
-        <v>4562</v>
-      </c>
-      <c r="G163" s="3" t="s">
-        <v>10</v>
+      <c r="F163" s="4">
+        <v>0</v>
+      </c>
+      <c r="G163" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="164" spans="1:7" x14ac:dyDescent="0.25">
@@ -5900,10 +5900,10 @@
         <v>120</v>
       </c>
       <c r="F164" s="4">
-        <v>264</v>
+        <v>0</v>
       </c>
       <c r="G164" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="165" spans="1:7" x14ac:dyDescent="0.25">
@@ -5922,11 +5922,11 @@
       <c r="E165">
         <v>120</v>
       </c>
-      <c r="F165" s="2">
-        <v>1260</v>
-      </c>
-      <c r="G165" s="3" t="s">
-        <v>10</v>
+      <c r="F165" s="4">
+        <v>0</v>
+      </c>
+      <c r="G165" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="166" spans="1:7" x14ac:dyDescent="0.25">
@@ -5945,11 +5945,11 @@
       <c r="E166">
         <v>120</v>
       </c>
-      <c r="F166" s="2">
-        <v>3735</v>
-      </c>
-      <c r="G166" s="3" t="s">
-        <v>10</v>
+      <c r="F166" s="4">
+        <v>0</v>
+      </c>
+      <c r="G166" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="167" spans="1:7" x14ac:dyDescent="0.25">
@@ -5968,11 +5968,11 @@
       <c r="E167">
         <v>120</v>
       </c>
-      <c r="F167" s="2">
-        <v>764</v>
-      </c>
-      <c r="G167" s="3" t="s">
-        <v>10</v>
+      <c r="F167" s="4">
+        <v>0</v>
+      </c>
+      <c r="G167" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="168" spans="1:7" x14ac:dyDescent="0.25">
@@ -5992,10 +5992,10 @@
         <v>120</v>
       </c>
       <c r="F168" s="4">
-        <v>157</v>
+        <v>0</v>
       </c>
       <c r="G168" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="169" spans="1:7" x14ac:dyDescent="0.25">
@@ -6014,11 +6014,11 @@
       <c r="E169">
         <v>120</v>
       </c>
-      <c r="F169" s="2">
-        <v>703</v>
-      </c>
-      <c r="G169" s="3" t="s">
-        <v>10</v>
+      <c r="F169" s="4">
+        <v>0</v>
+      </c>
+      <c r="G169" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="170" spans="1:7" x14ac:dyDescent="0.25">
@@ -6037,11 +6037,11 @@
       <c r="E170">
         <v>120</v>
       </c>
-      <c r="F170" s="6">
-        <v>0</v>
-      </c>
-      <c r="G170" s="7" t="s">
-        <v>23</v>
+      <c r="F170" s="4">
+        <v>0</v>
+      </c>
+      <c r="G170" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="171" spans="1:7" x14ac:dyDescent="0.25">
@@ -6060,11 +6060,11 @@
       <c r="E171">
         <v>120</v>
       </c>
-      <c r="F171" s="2">
-        <v>7702</v>
-      </c>
-      <c r="G171" s="3" t="s">
-        <v>10</v>
+      <c r="F171" s="4">
+        <v>0</v>
+      </c>
+      <c r="G171" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="172" spans="1:7" x14ac:dyDescent="0.25">
@@ -6083,11 +6083,11 @@
       <c r="E172">
         <v>120</v>
       </c>
-      <c r="F172" s="2">
-        <v>2089</v>
-      </c>
-      <c r="G172" s="3" t="s">
-        <v>10</v>
+      <c r="F172" s="4">
+        <v>0</v>
+      </c>
+      <c r="G172" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="173" spans="1:7" x14ac:dyDescent="0.25">
@@ -6106,11 +6106,11 @@
       <c r="E173">
         <v>1</v>
       </c>
-      <c r="F173" s="2">
-        <v>232</v>
-      </c>
-      <c r="G173" s="3" t="s">
-        <v>10</v>
+      <c r="F173" s="4">
+        <v>0</v>
+      </c>
+      <c r="G173" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="174" spans="1:7" x14ac:dyDescent="0.25">
@@ -6129,11 +6129,11 @@
       <c r="E174">
         <v>1</v>
       </c>
-      <c r="F174" s="2">
-        <v>147</v>
-      </c>
-      <c r="G174" s="3" t="s">
-        <v>10</v>
+      <c r="F174" s="4">
+        <v>0</v>
+      </c>
+      <c r="G174" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="175" spans="1:7" x14ac:dyDescent="0.25">
@@ -6153,10 +6153,10 @@
         <v>12</v>
       </c>
       <c r="F175" s="4">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="G175" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="176" spans="1:7" x14ac:dyDescent="0.25">
@@ -6175,11 +6175,11 @@
       <c r="E176">
         <v>12</v>
       </c>
-      <c r="F176" s="6">
-        <v>0</v>
-      </c>
-      <c r="G176" s="7" t="s">
-        <v>23</v>
+      <c r="F176" s="4">
+        <v>0</v>
+      </c>
+      <c r="G176" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="177" spans="1:7" x14ac:dyDescent="0.25">
@@ -6198,11 +6198,11 @@
       <c r="E177">
         <v>12</v>
       </c>
-      <c r="F177" s="6">
-        <v>0</v>
-      </c>
-      <c r="G177" s="7" t="s">
-        <v>23</v>
+      <c r="F177" s="4">
+        <v>0</v>
+      </c>
+      <c r="G177" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="178" spans="1:7" x14ac:dyDescent="0.25">
@@ -6221,11 +6221,11 @@
       <c r="E178">
         <v>12</v>
       </c>
-      <c r="F178" s="2">
-        <v>163</v>
-      </c>
-      <c r="G178" s="3" t="s">
-        <v>10</v>
+      <c r="F178" s="4">
+        <v>0</v>
+      </c>
+      <c r="G178" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="179" spans="1:7" x14ac:dyDescent="0.25">
@@ -6245,10 +6245,10 @@
         <v>12</v>
       </c>
       <c r="F179" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G179" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="180" spans="1:7" x14ac:dyDescent="0.25">
@@ -6267,11 +6267,11 @@
       <c r="E180">
         <v>12</v>
       </c>
-      <c r="F180" s="6">
-        <v>0</v>
-      </c>
-      <c r="G180" s="7" t="s">
-        <v>23</v>
+      <c r="F180" s="4">
+        <v>0</v>
+      </c>
+      <c r="G180" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="181" spans="1:7" x14ac:dyDescent="0.25">
@@ -6290,11 +6290,11 @@
       <c r="E181">
         <v>12</v>
       </c>
-      <c r="F181" s="6">
-        <v>0</v>
-      </c>
-      <c r="G181" s="7" t="s">
-        <v>23</v>
+      <c r="F181" s="4">
+        <v>0</v>
+      </c>
+      <c r="G181" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="182" spans="1:7" x14ac:dyDescent="0.25">
@@ -6313,11 +6313,11 @@
       <c r="E182">
         <v>12</v>
       </c>
-      <c r="F182" s="2">
-        <v>211</v>
-      </c>
-      <c r="G182" s="3" t="s">
-        <v>10</v>
+      <c r="F182" s="4">
+        <v>0</v>
+      </c>
+      <c r="G182" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="183" spans="1:7" x14ac:dyDescent="0.25">
@@ -6337,10 +6337,10 @@
         <v>12</v>
       </c>
       <c r="F183" s="4">
-        <v>53</v>
+        <v>0</v>
       </c>
       <c r="G183" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="184" spans="1:7" x14ac:dyDescent="0.25">
@@ -6360,10 +6360,10 @@
         <v>12</v>
       </c>
       <c r="F184" s="4">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="G184" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="185" spans="1:7" x14ac:dyDescent="0.25">
@@ -6382,11 +6382,11 @@
       <c r="E185">
         <v>12</v>
       </c>
-      <c r="F185" s="2">
-        <v>3022</v>
-      </c>
-      <c r="G185" s="3" t="s">
-        <v>10</v>
+      <c r="F185" s="4">
+        <v>0</v>
+      </c>
+      <c r="G185" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="186" spans="1:7" x14ac:dyDescent="0.25">
@@ -6405,11 +6405,11 @@
       <c r="E186">
         <v>12</v>
       </c>
-      <c r="F186" s="2">
-        <v>286</v>
-      </c>
-      <c r="G186" s="3" t="s">
-        <v>10</v>
+      <c r="F186" s="4">
+        <v>0</v>
+      </c>
+      <c r="G186" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="187" spans="1:7" x14ac:dyDescent="0.25">
@@ -6428,11 +6428,11 @@
       <c r="E187">
         <v>12</v>
       </c>
-      <c r="F187" s="2">
-        <v>157</v>
-      </c>
-      <c r="G187" s="3" t="s">
-        <v>10</v>
+      <c r="F187" s="4">
+        <v>0</v>
+      </c>
+      <c r="G187" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="188" spans="1:7" x14ac:dyDescent="0.25">
@@ -6451,11 +6451,11 @@
       <c r="E188">
         <v>12</v>
       </c>
-      <c r="F188" s="2">
-        <v>654</v>
-      </c>
-      <c r="G188" s="3" t="s">
-        <v>10</v>
+      <c r="F188" s="4">
+        <v>0</v>
+      </c>
+      <c r="G188" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="189" spans="1:7" x14ac:dyDescent="0.25">
@@ -6475,10 +6475,10 @@
         <v>18</v>
       </c>
       <c r="F189" s="4">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G189" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="190" spans="1:7" x14ac:dyDescent="0.25">
@@ -6497,11 +6497,11 @@
       <c r="E190">
         <v>12</v>
       </c>
-      <c r="F190" s="2">
-        <v>1156</v>
-      </c>
-      <c r="G190" s="3" t="s">
-        <v>10</v>
+      <c r="F190" s="4">
+        <v>0</v>
+      </c>
+      <c r="G190" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="191" spans="1:7" x14ac:dyDescent="0.25">
@@ -6520,11 +6520,11 @@
       <c r="E191">
         <v>18</v>
       </c>
-      <c r="F191" s="2">
-        <v>1901</v>
-      </c>
-      <c r="G191" s="3" t="s">
-        <v>10</v>
+      <c r="F191" s="4">
+        <v>0</v>
+      </c>
+      <c r="G191" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="192" spans="1:7" x14ac:dyDescent="0.25">
@@ -6543,11 +6543,11 @@
       <c r="E192">
         <v>12</v>
       </c>
-      <c r="F192" s="2">
-        <v>1913</v>
-      </c>
-      <c r="G192" s="3" t="s">
-        <v>10</v>
+      <c r="F192" s="4">
+        <v>0</v>
+      </c>
+      <c r="G192" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="193" spans="1:7" x14ac:dyDescent="0.25">
@@ -6566,11 +6566,11 @@
       <c r="E193">
         <v>400</v>
       </c>
-      <c r="F193" s="2">
-        <v>76950</v>
-      </c>
-      <c r="G193" s="3" t="s">
-        <v>10</v>
+      <c r="F193" s="4">
+        <v>0</v>
+      </c>
+      <c r="G193" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="194" spans="1:7" x14ac:dyDescent="0.25">
@@ -6589,11 +6589,11 @@
       <c r="E194">
         <v>400</v>
       </c>
-      <c r="F194" s="2">
-        <v>72165</v>
-      </c>
-      <c r="G194" s="3" t="s">
-        <v>10</v>
+      <c r="F194" s="4">
+        <v>0</v>
+      </c>
+      <c r="G194" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="195" spans="1:7" x14ac:dyDescent="0.25">
@@ -6612,11 +6612,11 @@
       <c r="E195">
         <v>120</v>
       </c>
-      <c r="F195" s="2">
-        <v>3620</v>
-      </c>
-      <c r="G195" s="3" t="s">
-        <v>10</v>
+      <c r="F195" s="4">
+        <v>0</v>
+      </c>
+      <c r="G195" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="196" spans="1:7" x14ac:dyDescent="0.25">
@@ -6635,11 +6635,11 @@
       <c r="E196">
         <v>120</v>
       </c>
-      <c r="F196" s="2">
-        <v>1816</v>
-      </c>
-      <c r="G196" s="3" t="s">
-        <v>10</v>
+      <c r="F196" s="4">
+        <v>0</v>
+      </c>
+      <c r="G196" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="197" spans="1:7" x14ac:dyDescent="0.25">
@@ -6658,11 +6658,11 @@
       <c r="E197">
         <v>120</v>
       </c>
-      <c r="F197" s="2">
-        <v>8964</v>
-      </c>
-      <c r="G197" s="3" t="s">
-        <v>10</v>
+      <c r="F197" s="4">
+        <v>0</v>
+      </c>
+      <c r="G197" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="198" spans="1:7" x14ac:dyDescent="0.25">
@@ -6681,11 +6681,11 @@
       <c r="E198">
         <v>120</v>
       </c>
-      <c r="F198" s="6">
-        <v>0</v>
-      </c>
-      <c r="G198" s="7" t="s">
-        <v>23</v>
+      <c r="F198" s="4">
+        <v>0</v>
+      </c>
+      <c r="G198" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="199" spans="1:7" x14ac:dyDescent="0.25">
@@ -6704,11 +6704,11 @@
       <c r="E199">
         <v>120</v>
       </c>
-      <c r="F199" s="2">
-        <v>8040</v>
-      </c>
-      <c r="G199" s="3" t="s">
-        <v>10</v>
+      <c r="F199" s="4">
+        <v>0</v>
+      </c>
+      <c r="G199" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>